<commit_message>
feat: analytics enhancement — surface unused measures, fix layout
Portfolio Overview:
  - Swap Completion Rate → YoY Growth % (trend metric belongs here)

Contract Lifecycle:
  - Add [Expiring Soon Value] as 5th KPI (AED exposure view)
  - Respace cards to 5×306w

Payment & Cashflow:
  - Add [MoM Growth %] as 5th KPI (trend direction at a glance)
  - Respace cards to 5×306w

Deliverables & Obligations:
  - Add [Deliverables Without Evidence] as 5th KPI (audit flag)
  - Respace cards to 5×306w

Season Analysis (hidden):
  - Add [Paid Amount] as 5th KPI (cash collected)
  - Fix tableEx out-of-bounds (h=290→246)

Counterparty & Relationship (hidden):
  - Respace cards to 5×306w
  - Fix tableEx out-of-bounds (h=290→246)

Compliance & Governance (hidden):
  - Fix 2× tableEx out-of-bounds (h=290→246)

All card rows aligned at y=158 for visual consistency.
</commit_message>
<xml_diff>
--- a/contracts_data_collection_template.xlsx
+++ b/contracts_data_collection_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dbln\code\powerbi-contract-uaepl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9074FAC3-B779-4046-8AE7-8E93716D1809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4245CED-1251-4134-BFCE-D13D56814AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24098" yWindow="-3450" windowWidth="24196" windowHeight="14475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1756" uniqueCount="680">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1757" uniqueCount="681">
   <si>
     <t>Contract Tracking Data Collection Template</t>
   </si>
@@ -2082,6 +2082,9 @@
   </si>
   <si>
     <t>AGR-2026-026</t>
+  </si>
+  <si>
+    <t>Testing</t>
   </si>
 </sst>
 </file>
@@ -2469,19 +2472,15 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -2493,6 +2492,10 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2599,14 +2602,14 @@
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="Unit" dataDxfId="7"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="Value_AED" dataDxfId="6"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="Frequency" dataDxfId="5"/>
-    <tableColumn id="20" xr3:uid="{0598B16E-6B1C-4C70-BF35-6F3BFEACC3EA}" name="Due" dataDxfId="0"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="Due_Date" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="Season" dataDxfId="3"/>
+    <tableColumn id="20" xr3:uid="{0598B16E-6B1C-4C70-BF35-6F3BFEACC3EA}" name="Due" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="Due_Date" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="Season" dataDxfId="2"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0200-00000D000000}" name="Owner"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0200-00000E000000}" name="Responsible_Party"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0200-00000F000000}" name="Applicable"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0200-000010000000}" name="Status" dataDxfId="2"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0200-000011000000}" name="Date_Delivered" dataDxfId="1"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0200-000010000000}" name="Status" dataDxfId="1"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0200-000011000000}" name="Date_Delivered" dataDxfId="0"/>
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0200-000012000000}" name="Evidence_Link"/>
     <tableColumn id="19" xr3:uid="{00000000-0010-0000-0200-000013000000}" name="Notes"/>
   </tableColumns>
@@ -2813,16 +2816,16 @@
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:H23"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="44" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="53.8125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.8125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.8125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="53.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.796875" bestFit="1" customWidth="1"/>
     <col min="5" max="8" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="20.65">
+    <row r="1" spans="1:8" ht="21">
       <c r="A1" s="52" t="s">
         <v>0</v>
       </c>
@@ -2844,7 +2847,7 @@
       <c r="G2" s="53"/>
       <c r="H2" s="53"/>
     </row>
-    <row r="4" spans="1:8" ht="13.9">
+    <row r="4" spans="1:8">
       <c r="A4" s="27" t="s">
         <v>1</v>
       </c>
@@ -2962,8 +2965,8 @@
       <c r="C12" s="31"/>
       <c r="D12" s="31"/>
     </row>
-    <row r="13" spans="1:8" ht="13.9">
-      <c r="A13" s="56" t="s">
+    <row r="13" spans="1:8">
+      <c r="A13" s="55" t="s">
         <v>30</v>
       </c>
       <c r="B13" s="53"/>
@@ -2975,40 +2978,40 @@
       <c r="H13" s="53"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="55" t="s">
+      <c r="A14" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="55"/>
-      <c r="C14" s="55"/>
-      <c r="D14" s="55"/>
-      <c r="E14" s="55"/>
-      <c r="F14" s="55"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
+      <c r="B14" s="56"/>
+      <c r="C14" s="56"/>
+      <c r="D14" s="56"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="56"/>
+      <c r="G14" s="56"/>
+      <c r="H14" s="56"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="55" t="s">
+      <c r="A15" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="55"/>
-      <c r="C15" s="55"/>
-      <c r="D15" s="55"/>
-      <c r="E15" s="55"/>
-      <c r="F15" s="55"/>
-      <c r="G15" s="55"/>
-      <c r="H15" s="55"/>
+      <c r="B15" s="56"/>
+      <c r="C15" s="56"/>
+      <c r="D15" s="56"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="56"/>
+      <c r="G15" s="56"/>
+      <c r="H15" s="56"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="55"/>
-      <c r="B16" s="55"/>
-      <c r="C16" s="55"/>
-      <c r="D16" s="55"/>
-      <c r="E16" s="55"/>
-      <c r="F16" s="55"/>
-      <c r="G16" s="55"/>
-      <c r="H16" s="55"/>
-    </row>
-    <row r="18" spans="1:8" ht="19.149999999999999" customHeight="1">
+      <c r="A16" s="56"/>
+      <c r="B16" s="56"/>
+      <c r="C16" s="56"/>
+      <c r="D16" s="56"/>
+      <c r="E16" s="56"/>
+      <c r="F16" s="56"/>
+      <c r="G16" s="56"/>
+      <c r="H16" s="56"/>
+    </row>
+    <row r="18" spans="1:8" ht="19.2" customHeight="1">
       <c r="A18" s="52" t="s">
         <v>33</v>
       </c>
@@ -3032,7 +3035,7 @@
       <c r="G19" s="54"/>
       <c r="H19" s="54"/>
     </row>
-    <row r="20" spans="1:8" ht="19.149999999999999" customHeight="1">
+    <row r="20" spans="1:8" ht="19.2" customHeight="1">
       <c r="A20" s="52" t="s">
         <v>89</v>
       </c>
@@ -3056,7 +3059,7 @@
       <c r="G21" s="53"/>
       <c r="H21" s="53"/>
     </row>
-    <row r="22" spans="1:8" ht="19.149999999999999" customHeight="1">
+    <row r="22" spans="1:8" ht="19.2" customHeight="1">
       <c r="A22" s="52" t="s">
         <v>118</v>
       </c>
@@ -3082,11 +3085,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A15:H15"/>
     <mergeCell ref="A22:H22"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A16:H16"/>
@@ -3094,6 +3092,11 @@
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A15:H15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3105,29 +3108,37 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:AC201"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="20.5" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="1" max="1" width="15.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.19921875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="11" width="18" customWidth="1"/>
-    <col min="12" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="27.5625" customWidth="1"/>
-    <col min="16" max="16" width="12" customWidth="1"/>
-    <col min="17" max="18" width="18" customWidth="1"/>
-    <col min="19" max="19" width="20.625" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="15" customWidth="1"/>
-    <col min="22" max="22" width="18.9375" customWidth="1"/>
-    <col min="23" max="23" width="20" customWidth="1"/>
-    <col min="24" max="24" width="16" customWidth="1"/>
-    <col min="25" max="25" width="34" customWidth="1"/>
-    <col min="26" max="27" width="16" customWidth="1"/>
-    <col min="28" max="28" width="30" customWidth="1"/>
-    <col min="29" max="29" width="34" customWidth="1"/>
+    <col min="5" max="5" width="20.19921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.8984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.19921875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.3984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="27.796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="26.69921875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="21.296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.69921875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20.796875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="21.69921875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.8984375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.69921875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="21.59765625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18.69921875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="53.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="15" customHeight="1">
@@ -10802,10 +10813,24 @@
       <c r="AC201" s="4"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="whole" sqref="V2:V201" xr:uid="{00000000-0002-0000-0100-000007000000}">
+  <dataValidations count="6">
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Please add a valid date" sqref="AA1:AA1048576" xr:uid="{A445C817-ACFD-4535-B3F6-8DF9C1D10D02}">
+      <formula1>36526</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Please enter a valid data" sqref="Z1:Z1048576" xr:uid="{67DB9211-F369-48AC-8189-C406645C2783}">
+      <formula1>36526</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Accepted format ARG-000-000" error="Accepted format ARG-000-000" promptTitle="Accepted format ARG-000-000" sqref="A1:A1048576" xr:uid="{968FFE82-1574-4CBC-B069-9E0C6EE14F47}">
+      <formula1>"'=AND(LEFT(A2:A200,4)=""AGR-"",LEN(A2:200)=10,COUNTIF($A$2:$A$1000,A2)&lt;=1)"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N1:N1048576" xr:uid="{75EBE032-DF89-4F7B-A173-050ABFDE9D54}">
       <formula1>0</formula1>
-      <formula2>365</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q1:Q1048576 R1:R1048576" xr:uid="{4196957B-C7E0-43E3-A1B1-9B5CEC7AF497}">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V1:V1048576" xr:uid="{1538F1F5-92CB-442D-B585-F1348CC6A84A}">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10815,24 +10840,6 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="10">
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000000000000}">
-          <x14:formula1>
-            <xm:f>Lookups!$A$5:$A$9</xm:f>
-          </x14:formula1>
-          <xm:sqref>B5:B201 B3</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000001000000}">
-          <x14:formula1>
-            <xm:f>Lookups!$B$5:$B$10</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2:D201</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000002000000}">
-          <x14:formula1>
-            <xm:f>Lookups!$C$5:$C$11</xm:f>
-          </x14:formula1>
-          <xm:sqref>G2:G201</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000003000000}">
           <x14:formula1>
             <xm:f>Lookups!$D$5:$D$12</xm:f>
@@ -10845,35 +10852,53 @@
           </x14:formula1>
           <xm:sqref>P2:P201</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000005000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{158B5955-4D29-4B9A-A580-95360E1E2441}">
           <x14:formula1>
-            <xm:f>Lookups!$F$5:$F$11</xm:f>
+            <xm:f>Lookups!$G$5:$G$17</xm:f>
           </x14:formula1>
-          <xm:sqref>S2:S201</xm:sqref>
+          <xm:sqref>T1:T1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000006000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{327E2DE2-0126-471F-B201-AA74182344D5}">
           <x14:formula1>
-            <xm:f>Lookups!$G$5:$G$7</xm:f>
+            <xm:f>Lookups!$A$5:$A$17</xm:f>
           </x14:formula1>
-          <xm:sqref>T2:U201</xm:sqref>
+          <xm:sqref>B1:B1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000008000000}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{25A52713-5D5F-448F-BDBE-A358E5B2E7B4}">
           <x14:formula1>
-            <xm:f>Lookups!$H$5:$H$8</xm:f>
+            <xm:f>Lookups!$B$5:$B$18</xm:f>
           </x14:formula1>
-          <xm:sqref>W2:W201</xm:sqref>
+          <xm:sqref>D1:D1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" errorStyle="warning" showErrorMessage="1" xr:uid="{B5BF129E-5A51-4FEB-AF92-DD962CD583C8}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2E15B959-EDCA-4488-B851-691A73A38930}">
           <x14:formula1>
-            <xm:f>Lookups!$A$5:$A$9</xm:f>
+            <xm:f>Lookups!$C$5:$C$18</xm:f>
           </x14:formula1>
-          <xm:sqref>B4</xm:sqref>
+          <xm:sqref>G1:G1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" showErrorMessage="1" xr:uid="{94CEFF77-89DB-492C-B1EB-7619B8807729}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{538281CC-4972-40AB-9053-2D19AE77261A}">
           <x14:formula1>
-            <xm:f>Lookups!$A$5:$A$9</xm:f>
+            <xm:f>Lookups!$M$5:$M$18</xm:f>
           </x14:formula1>
-          <xm:sqref>B2</xm:sqref>
+          <xm:sqref>H1:H1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D088664F-7493-4DD6-84EA-73B19AA325EC}">
+          <x14:formula1>
+            <xm:f>Lookups!$F$5:$F$18</xm:f>
+          </x14:formula1>
+          <xm:sqref>S1:S1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8DF4B97F-01CA-4C5C-9AB2-449570BC7D93}">
+          <x14:formula1>
+            <xm:f>Lookups!$G$5:$G$18</xm:f>
+          </x14:formula1>
+          <xm:sqref>U1:U1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7CF738EA-2DD6-444C-9493-D06F928DA0EB}">
+          <x14:formula1>
+            <xm:f>Lookups!$H$5:$H$18</xm:f>
+          </x14:formula1>
+          <xm:sqref>W1:W1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -10887,25 +10912,25 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:P401"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="15.3125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5625" style="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.59765625" style="34" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.8125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.4375" customWidth="1"/>
-    <col min="7" max="7" width="11.5625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.3984375" customWidth="1"/>
+    <col min="7" max="7" width="11.59765625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.5625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.59765625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.5625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.0625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.19921875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.59765625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.09765625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.25" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="39.25" customWidth="1"/>
-    <col min="17" max="17" width="18.8125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.19921875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="39.19921875" customWidth="1"/>
+    <col min="17" max="17" width="18.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15" customHeight="1">
@@ -10997,7 +11022,7 @@
       </c>
       <c r="O2" s="4">
         <f t="shared" ref="O2:O65" ca="1" si="0">IF(A2="","",IF(G2="","",G2-TODAY()))</f>
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="P2" s="4"/>
     </row>
@@ -11040,7 +11065,7 @@
       </c>
       <c r="O3" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>523</v>
+        <v>513</v>
       </c>
       <c r="P3" s="4"/>
     </row>
@@ -11083,7 +11108,7 @@
       </c>
       <c r="O4" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>889</v>
+        <v>879</v>
       </c>
       <c r="P4" s="4"/>
     </row>
@@ -11126,7 +11151,7 @@
       </c>
       <c r="O5" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>-118</v>
+        <v>-128</v>
       </c>
       <c r="P5" s="4"/>
     </row>
@@ -11212,7 +11237,7 @@
       </c>
       <c r="O7" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>339</v>
+        <v>329</v>
       </c>
       <c r="P7" s="4"/>
     </row>
@@ -11255,7 +11280,7 @@
       </c>
       <c r="O8" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>675</v>
+        <v>665</v>
       </c>
       <c r="P8" s="4"/>
     </row>
@@ -11296,7 +11321,7 @@
       <c r="N9" s="4"/>
       <c r="O9" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>-74</v>
+        <v>-84</v>
       </c>
       <c r="P9" s="4"/>
     </row>
@@ -11337,7 +11362,7 @@
       <c r="N10" s="4"/>
       <c r="O10" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="P10" s="4"/>
     </row>
@@ -11378,7 +11403,7 @@
       <c r="N11" s="4"/>
       <c r="O11" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>675</v>
+        <v>665</v>
       </c>
       <c r="P11" s="4"/>
     </row>
@@ -19574,10 +19599,25 @@
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
-  <dataValidations count="1">
-    <dataValidation type="whole" sqref="C2:C401" xr:uid="{00000000-0002-0000-0200-000001000000}">
+  <dataValidations count="6">
+    <dataValidation type="whole" sqref="C1:C1048576" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>1</formula1>
       <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K1:K1048576" xr:uid="{ED054E36-A2A9-4FBB-AFB4-78044E7F0559}">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1:L1048576" xr:uid="{CC796EDF-5920-45BB-BA06-8D5306D1F3C2}">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1:I1048576" xr:uid="{0273EF36-C5E6-4B9C-AAE2-E8119800BD3F}">
+      <formula1>36526</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O1:O1048576" xr:uid="{89121B33-08D6-4A58-9B42-0C140E0377B5}">
+      <formula1>-10000</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A1195" xr:uid="{C063BD5A-D919-448B-84EE-B699C84CA670}">
+      <formula1>AND(LEFT(A2,4)="PAY-",LEN(A2)=15,COUNTIF($A$2:$A$1000,A2)&lt;=1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -19587,29 +19627,29 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0200-000000000000}">
-          <x14:formula1>
-            <xm:f>Agreements!$A$2:$A$201</xm:f>
-          </x14:formula1>
-          <xm:sqref>B2:B401</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0200-000002000000}">
-          <x14:formula1>
-            <xm:f>Lookups!$J$5:$J$10</xm:f>
-          </x14:formula1>
-          <xm:sqref>E2:E401</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0200-000003000000}">
           <x14:formula1>
             <xm:f>Lookups!$E$5:$E$10</xm:f>
           </x14:formula1>
           <xm:sqref>J2:J401</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0200-000004000000}">
+        <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" xr:uid="{392E73CF-4333-4A7B-9B07-4A2078427585}">
           <x14:formula1>
-            <xm:f>Lookups!$I$5:$I$12</xm:f>
+            <xm:f>Lookups!$I$5:$I$18</xm:f>
           </x14:formula1>
-          <xm:sqref>N2:N401</xm:sqref>
+          <xm:sqref>N1:N1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" xr:uid="{02602F3E-DB2E-4AEA-827B-0627007653CC}">
+          <x14:formula1>
+            <xm:f>Lookups!$J$5:$J$18</xm:f>
+          </x14:formula1>
+          <xm:sqref>E1:E1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D72BBBCB-EF8E-4D02-A87B-69D54A1D4E5D}">
+          <x14:formula1>
+            <xm:f>Agreements!$A$2:$A$201</xm:f>
+          </x14:formula1>
+          <xm:sqref>B1:B1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -19623,26 +19663,28 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:T497"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="18.09765625" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="40.25" customWidth="1"/>
-    <col min="6" max="6" width="90.4375" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="14" style="34" customWidth="1"/>
-    <col min="9" max="9" width="18.5625" style="34" customWidth="1"/>
-    <col min="10" max="10" width="19.9375" style="34" customWidth="1"/>
-    <col min="11" max="11" width="21" customWidth="1"/>
-    <col min="12" max="12" width="15.3125" customWidth="1"/>
-    <col min="13" max="13" width="18" customWidth="1"/>
-    <col min="14" max="14" width="24.3125" customWidth="1"/>
-    <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="16" width="18" style="34" customWidth="1"/>
-    <col min="17" max="17" width="16" customWidth="1"/>
-    <col min="18" max="20" width="34" customWidth="1"/>
+    <col min="1" max="1" width="15.8984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.09765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="64.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="103.3984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.59765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.3984375" style="34" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.296875" style="34" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.5" style="34" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.69921875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.69921875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.296875" style="34" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.09765625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="8.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="15" customHeight="1">
@@ -32948,60 +32990,80 @@
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
+  <dataValidations count="4">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1:I1048576" xr:uid="{0771FC39-4EF5-434E-91DC-A2FA1E9B6F2A}">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1:G1048576" xr:uid="{9E3D272D-E53D-4D44-A88B-344CF9D20C8F}">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1:L1048576" xr:uid="{92B462D2-8C01-4DB1-B702-5F98A593AB7D}">
+      <formula1>36526</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R1:R1048576" xr:uid="{687D3C41-A8C9-4EA1-9774-72AB80247DEB}">
+      <formula1>36526</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8">
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0300-000000000000}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="9">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0300-000000000000}">
           <x14:formula1>
             <xm:f>Agreements!$A$2:$A$201</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B497</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0300-000001000000}">
-          <x14:formula1>
-            <xm:f>Lookups!$K$5:$K$12</xm:f>
-          </x14:formula1>
-          <xm:sqref>C2:C497</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0300-000002000000}">
-          <x14:formula1>
-            <xm:f>Lookups!$L$5:$L$15</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2:D497</xm:sqref>
+          <xm:sqref>B1:B1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0300-000003000000}">
           <x14:formula1>
             <xm:f>Lookups!$O$5:$O$18</xm:f>
           </x14:formula1>
-          <xm:sqref>H2:H497</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0300-000004000000}">
-          <x14:formula1>
-            <xm:f>Lookups!$M$5:$M$13</xm:f>
-          </x14:formula1>
-          <xm:sqref>N2:N497</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0300-000005000000}">
-          <x14:formula1>
-            <xm:f>Lookups!$N$5:$N$10</xm:f>
-          </x14:formula1>
-          <xm:sqref>O2:O497</xm:sqref>
+          <xm:sqref>H1:H1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0300-000006000000}">
           <x14:formula1>
             <xm:f>Lookups!$G$5:$G$7</xm:f>
           </x14:formula1>
-          <xm:sqref>P2:P497</xm:sqref>
+          <xm:sqref>P1:P1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0300-000007000000}">
           <x14:formula1>
             <xm:f>Lookups!$P$5:$P$11</xm:f>
           </x14:formula1>
           <xm:sqref>Q2:Q497</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{254F4B4A-B2DF-4EAA-B8AC-DEFCD0AFB9EC}">
+          <x14:formula1>
+            <xm:f>Lookups!$F$5:$F$18</xm:f>
+          </x14:formula1>
+          <xm:sqref>J1:J1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C3331441-3DE0-4B9C-AF6D-C3D828A405F9}">
+          <x14:formula1>
+            <xm:f>Lookups!$K$5:$K$18</xm:f>
+          </x14:formula1>
+          <xm:sqref>C1:C1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{CF90D3A7-E1EA-4719-B94B-8D22507CEE54}">
+          <x14:formula1>
+            <xm:f>Lookups!$L$5:$L$18</xm:f>
+          </x14:formula1>
+          <xm:sqref>D1:D1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" xr:uid="{7BAF3703-D0F4-4B78-BC91-C35C2E5C1E42}">
+          <x14:formula1>
+            <xm:f>Lookups!$M$5:$M$18</xm:f>
+          </x14:formula1>
+          <xm:sqref>N1:N1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" xr:uid="{C454803E-A72D-4A12-A570-E3E21642979D}">
+          <x14:formula1>
+            <xm:f>Lookups!$N$5:$N$18</xm:f>
+          </x14:formula1>
+          <xm:sqref>O1:O1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -33015,14 +33077,14 @@
     <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="19.149999999999999" customHeight="1">
+    <row r="1" spans="1:8" ht="19.2" customHeight="1">
       <c r="A1" s="52" t="s">
         <v>174</v>
       </c>
@@ -33216,7 +33278,7 @@
     <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:H42"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -33227,7 +33289,7 @@
     <col min="7" max="7" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="19.149999999999999" customHeight="1">
+    <row r="1" spans="1:8" ht="19.2" customHeight="1">
       <c r="A1" s="52" t="s">
         <v>201</v>
       </c>
@@ -34163,12 +34225,12 @@
     <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:P18"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="16" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="19.149999999999999" customHeight="1">
+    <row r="1" spans="1:16" ht="19.2" customHeight="1">
       <c r="A1" s="52" t="s">
         <v>315</v>
       </c>
@@ -34475,7 +34537,9 @@
       </c>
     </row>
     <row r="10" spans="1:16" ht="15" customHeight="1">
-      <c r="A10" s="8"/>
+      <c r="A10" s="8" t="s">
+        <v>680</v>
+      </c>
       <c r="B10" s="9" t="s">
         <v>350</v>
       </c>

</xml_diff>

<commit_message>
fix: remove Zone.Identifier files and normalize SharePoint ApiVersion
- Deleted :Zone.Identifier files from PBIP project (colon in filename
  violates OPC URI rules, causing 'Part URI is not valid' error on publish
  and 'file path invalid' on save-as-PBIX)
- Updated .gitignore pattern from *:Zone.Identifier to **Zone.Identifier
- Normalized Agreements SharePoint ApiVersion from 15 to 'Auto' to match
  Deliverables and Payments tables
</commit_message>
<xml_diff>
--- a/contracts_data_collection_template.xlsx
+++ b/contracts_data_collection_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dbln\code\powerbi-contract-uaepl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4245CED-1251-4134-BFCE-D13D56814AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E4F645-01BB-491A-8D15-98C5F8BC9BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -2472,10 +2472,10 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2966,7 +2966,7 @@
       <c r="D12" s="31"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="55" t="s">
+      <c r="A13" s="56" t="s">
         <v>30</v>
       </c>
       <c r="B13" s="53"/>
@@ -2978,38 +2978,38 @@
       <c r="H13" s="53"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="56" t="s">
+      <c r="A14" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="56"/>
-      <c r="C14" s="56"/>
-      <c r="D14" s="56"/>
-      <c r="E14" s="56"/>
-      <c r="F14" s="56"/>
-      <c r="G14" s="56"/>
-      <c r="H14" s="56"/>
+      <c r="B14" s="55"/>
+      <c r="C14" s="55"/>
+      <c r="D14" s="55"/>
+      <c r="E14" s="55"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="56" t="s">
+      <c r="A15" s="55" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="56"/>
-      <c r="C15" s="56"/>
-      <c r="D15" s="56"/>
-      <c r="E15" s="56"/>
-      <c r="F15" s="56"/>
-      <c r="G15" s="56"/>
-      <c r="H15" s="56"/>
+      <c r="B15" s="55"/>
+      <c r="C15" s="55"/>
+      <c r="D15" s="55"/>
+      <c r="E15" s="55"/>
+      <c r="F15" s="55"/>
+      <c r="G15" s="55"/>
+      <c r="H15" s="55"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="56"/>
-      <c r="B16" s="56"/>
-      <c r="C16" s="56"/>
-      <c r="D16" s="56"/>
-      <c r="E16" s="56"/>
-      <c r="F16" s="56"/>
-      <c r="G16" s="56"/>
-      <c r="H16" s="56"/>
+      <c r="A16" s="55"/>
+      <c r="B16" s="55"/>
+      <c r="C16" s="55"/>
+      <c r="D16" s="55"/>
+      <c r="E16" s="55"/>
+      <c r="F16" s="55"/>
+      <c r="G16" s="55"/>
+      <c r="H16" s="55"/>
     </row>
     <row r="18" spans="1:8" ht="19.2" customHeight="1">
       <c r="A18" s="52" t="s">
@@ -3085,6 +3085,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A15:H15"/>
     <mergeCell ref="A22:H22"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A16:H16"/>
@@ -3092,11 +3097,6 @@
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A15:H15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10813,24 +10813,21 @@
       <c r="AC201" s="4"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="5">
     <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Please add a valid date" sqref="AA1:AA1048576" xr:uid="{A445C817-ACFD-4535-B3F6-8DF9C1D10D02}">
       <formula1>36526</formula1>
     </dataValidation>
     <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Please enter a valid data" sqref="Z1:Z1048576" xr:uid="{67DB9211-F369-48AC-8189-C406645C2783}">
       <formula1>36526</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Accepted format ARG-000-000" error="Accepted format ARG-000-000" promptTitle="Accepted format ARG-000-000" sqref="A1:A1048576" xr:uid="{968FFE82-1574-4CBC-B069-9E0C6EE14F47}">
-      <formula1>"'=AND(LEFT(A2:A200,4)=""AGR-"",LEN(A2:200)=10,COUNTIF($A$2:$A$1000,A2)&lt;=1)"</formula1>
-    </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N1:N1048576" xr:uid="{75EBE032-DF89-4F7B-A173-050ABFDE9D54}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N1:N1048576 V1:V1048576" xr:uid="{75EBE032-DF89-4F7B-A173-050ABFDE9D54}">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q1:Q1048576 R1:R1048576" xr:uid="{4196957B-C7E0-43E3-A1B1-9B5CEC7AF497}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V1:V1048576" xr:uid="{1538F1F5-92CB-442D-B585-F1348CC6A84A}">
-      <formula1>0</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A200" xr:uid="{CF09C8A3-05E8-4D8C-B20F-3A9FD5099A4E}">
+      <formula1>LEFT(A2,4)="AGR-"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11022,7 +11019,7 @@
       </c>
       <c r="O2" s="4">
         <f t="shared" ref="O2:O65" ca="1" si="0">IF(A2="","",IF(G2="","",G2-TODAY()))</f>
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="P2" s="4"/>
     </row>
@@ -11065,7 +11062,7 @@
       </c>
       <c r="O3" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="P3" s="4"/>
     </row>
@@ -11108,7 +11105,7 @@
       </c>
       <c r="O4" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="P4" s="4"/>
     </row>
@@ -11151,7 +11148,7 @@
       </c>
       <c r="O5" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>-128</v>
+        <v>-129</v>
       </c>
       <c r="P5" s="4"/>
     </row>
@@ -11237,7 +11234,7 @@
       </c>
       <c r="O7" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="P7" s="4"/>
     </row>
@@ -11280,7 +11277,7 @@
       </c>
       <c r="O8" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="P8" s="4"/>
     </row>
@@ -11321,7 +11318,7 @@
       <c r="N9" s="4"/>
       <c r="O9" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>-84</v>
+        <v>-85</v>
       </c>
       <c r="P9" s="4"/>
     </row>
@@ -11362,7 +11359,7 @@
       <c r="N10" s="4"/>
       <c r="O10" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="P10" s="4"/>
     </row>
@@ -11403,7 +11400,7 @@
       <c r="N11" s="4"/>
       <c r="O11" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="P11" s="4"/>
     </row>
@@ -19604,10 +19601,7 @@
       <formula1>1</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K1:K1048576" xr:uid="{ED054E36-A2A9-4FBB-AFB4-78044E7F0559}">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L1:L1048576" xr:uid="{CC796EDF-5920-45BB-BA06-8D5306D1F3C2}">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K1:L1048576" xr:uid="{ED054E36-A2A9-4FBB-AFB4-78044E7F0559}">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1:I1048576" xr:uid="{0273EF36-C5E6-4B9C-AAE2-E8119800BD3F}">
@@ -19616,8 +19610,11 @@
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O1:O1048576" xr:uid="{89121B33-08D6-4A58-9B42-0C140E0377B5}">
       <formula1>-10000</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A1195" xr:uid="{C063BD5A-D919-448B-84EE-B699C84CA670}">
-      <formula1>AND(LEFT(A2,4)="PAY-",LEN(A2)=15,COUNTIF($A$2:$A$1000,A2)&lt;=1)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A401" xr:uid="{F2F9FBF9-385D-423D-9EB3-055857BB97ED}">
+      <formula1>LEFT(A2,4)="PAY-"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1 A402:A1048576" xr:uid="{C063BD5A-D919-448B-84EE-B699C84CA670}">
+      <formula1>AND(LEFT(A1,4)="PAY-",LEN(A1)=15,COUNTIF($A$2:$A$1000,A1)&lt;=1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -32990,7 +32987,7 @@
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1:I1048576" xr:uid="{0771FC39-4EF5-434E-91DC-A2FA1E9B6F2A}">
       <formula1>0</formula1>
     </dataValidation>
@@ -33002,6 +32999,9 @@
     </dataValidation>
     <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R1:R1048576" xr:uid="{687D3C41-A8C9-4EA1-9774-72AB80247DEB}">
       <formula1>36526</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A497" xr:uid="{2282A9C5-035F-4B65-A368-E18C9EE0B9CD}">
+      <formula1>LEFT(A2,4)="ITM-"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>